<commit_message>
Reference the published Google Sheet in the Research Summary
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LegalReach_US_IP_Firms_Research.xlsx
+++ b/LegalReach_US_IP_Firms_Research.xlsx
@@ -6179,7 +6179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -6360,22 +6360,34 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Method</t>
+          <t>Google Sheet (same six tabs, live)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Every one of the 9 directory pages was read directly. Each listing's website was taken (a) from the Legal Reach profile text where the site publishes one, (b) from a cross-check against the firm's LegalServicesLink profile already extracted in this project, or (c) from a name + city web search whose result matched the listed address/phone. No URL was guessed; where nothing verifiable was found the cell is blank.</t>
+          <t>https://docs.google.com/spreadsheets/d/1GdoyB8__oIs76oh7yYXFoJT9END07cRB7lYppk1Yc5E/edit</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Every one of the 9 directory pages was read directly. Each listing's website was taken (a) from the Legal Reach profile text where the site publishes one, (b) from a cross-check against the firm's LegalServicesLink profile already extracted in this project, or (c) from a name + city web search whose result matched the listed address/phone. No URL was guessed; where nothing verifiable was found the cell is blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Caveats</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Legal Reach mixes firms, solo attorneys and extra office listings, and it also carries a few non-US firms. Two listings (Verhagen Bennett, Long and Associates) carry status notes worth a manual look.</t>
         </is>

</xml_diff>